<commit_message>
[Test] MS ThirdParty Admins Notifications Users
</commit_message>
<xml_diff>
--- a/src/__tests__/thirdParties/web/__testFiles__/Codigos_municipios_DANE.xlsx
+++ b/src/__tests__/thirdParties/web/__testFiles__/Codigos_municipios_DANE.xlsx
@@ -8,17 +8,26 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Proyectos\cali-mobility\cali-mobility-backend\src\__tests__\thirdParties\web\__testFiles__\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D3518EE-6174-4AD9-9719-F9C5DB351064}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58F568B9-41C5-414C-99F0-9CCBC7E72DCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21390" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -89,10 +98,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -413,7 +423,7 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2">
+      <c r="A2" s="3">
         <v>9991</v>
       </c>
       <c r="B2" s="1" t="s">
@@ -424,7 +434,7 @@
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3">
+      <c r="A3" s="3">
         <v>9992</v>
       </c>
       <c r="B3" s="1" t="s">
@@ -435,7 +445,7 @@
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4">
+      <c r="A4" s="3">
         <v>9993</v>
       </c>
       <c r="B4" s="1" t="s">

</xml_diff>